<commit_message>
Preenche planilha e dados de exemplo com o relatório de referência
Textos completos de análise por editoria (Jornalismo, Dramaturgia,
Institucional, Variedades, Esportes, Especiais), metodologia integral e
demais tabelas extraídos do PPTX Elife da semana 29/06–05/07.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planilha_Dash_Semanal_Globo.xlsx
+++ b/Planilha_Dash_Semanal_Globo.xlsx
@@ -68,10 +68,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -447,8 +453,8 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,12 +488,12 @@
           <t>VAR_MEDIA_3M_PCT</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>MEDIA_3M_INFO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>INSIGHT_SEMANA</t>
         </is>
@@ -524,12 +530,12 @@
           <t>-92%</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>(média diária/últimos 3 meses; comparação apenas em X) 783.417 (24/02–24/05)</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Jogo da Copa do Mundo entre Brasil e Noruega elevou o buzz.</t>
         </is>
@@ -551,7 +557,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -788,7 +794,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>quem ama cuida</t>
+          <t>hoje tem novela / quem ama cuida</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -812,7 +818,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -899,7 +905,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JN: Venezuelano que passou 4 dias soterrado conta que foi o único encontrado vivo</t>
+          <t>JN: Venezuelano que passou 4 dias soterrado conta que foi o único encontrado vivo em prédio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -930,7 +936,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -944,7 +950,7 @@
           <t>EDITORIA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>HEADLINE</t>
         </is>
@@ -961,9 +967,9 @@
           <t>Jornalismo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Jornalismo</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Jornal Nacional liderou em volume absoluto, enquanto Fantástico e Jornal da Globo dobraram seu alcance em meio a cobranças sobre o STF e polêmicas envolvendo Flávio Bolsonaro</t>
         </is>
       </c>
     </row>
@@ -978,9 +984,9 @@
           <t>Dramaturgia</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Dramaturgia</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Quem Ama Cuida atingiu 117 mil depoimentos liderada por memes de Letícia Colin, enquanto Coração Acelerado cresceu com evento sertanejo em Goiânia e A Nobreza do Amor foi celebrada após anúncio de Taís Araújo no elenco</t>
         </is>
       </c>
     </row>
@@ -992,12 +998,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Variedades</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Variedades</t>
+          <t>Institucional</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Provocação da Cazé TV ganhou tração e puxou volume de menções à Globo; atuação de Cristiane como comentarista foi o contraponto positivo</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1015,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Esportes</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Esportes</t>
+          <t>Variedades</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Especial de "Rei do Gado" fez Viver Sertanejo saltar 478%, enquanto Domingão repercutiu com a eliminação do Brasil e polêmicas</t>
         </is>
       </c>
     </row>
@@ -1026,12 +1032,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Institucional</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Institucional</t>
+          <t>Esportes</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>#CopaÉNaGlobo! Comentário de Ana Thaís Matos sobre Neymar dividiu opiniões durante a eliminação para a Noruega</t>
         </is>
       </c>
     </row>
@@ -1046,9 +1052,9 @@
           <t>Especiais</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Headline (frase de destaque em verde) da editoria Especiais</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Solidariedade a Luís Roberto marcou os esportes; Sessão da Tarde e Som Brasil completaram a semana</t>
         </is>
       </c>
     </row>
@@ -1063,13 +1069,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1088,7 +1094,7 @@
           <t>PROGRAMA_TAG</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>TEXTO</t>
         </is>
@@ -1110,9 +1116,9 @@
           <t>#JornalNacional</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>alcançou 30,4 mil depoimentos. Texto de análise do programa.</t>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>alcançou 30,4 mil depoimentos. A repercussão dos assuntos desta semana se concentrou em debates politizados. Um internauta somou 7,1 mil interações ao induzir que o JN estaria sendo favorável ao espectro político de direita ao não noticiar aquisições do senador Flávio Bolsonaro. Em especial, a matéria que informou o posicionamento do governo dos EUA ao considerar o PCC como a maior organização criminosa transnacional do Hemisfério Ocidental se fez presente em grande parte das menções informativas.</t>
         </is>
       </c>
     </row>
@@ -1132,9 +1138,9 @@
           <t>#Fantástico</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>gerou 15,3 mil depoimentos, crescimento de 140%.</t>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>gerou 16,3 mil depoimentos, resultando em 140% de crescimento em comparação à semana passada. O público, incluindo o deputado federal Nikolas Ferreira, repercutiu e cobrou uma matéria no Fantástico sobre as conversas vazadas entre Viviane Barci, esposa de Alexandre de Moraes, e Daniel Vorcaro, envolvendo uma minuta de contrato de R$129 milhões em honorários por serviços prestados ao Banco Master. Já a entrevista do goleiro Alisson Becker no programa gerou lamentações nas redes sociais pela eliminação do Brasil na Copa do Mundo.</t>
         </is>
       </c>
     </row>
@@ -1146,17 +1152,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dramaturgia</t>
+          <t>Jornalismo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>#QuemAmaCuida</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>obteve 117,4 mil depoimentos, 37% de crescimento.</t>
+          <t>#JornaldaGlobo</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>somou 7,3 mil depoimentos, atingindo um crescimento de 97% em relação à semana anterior. Duas matérias concentraram a maior repercussão nas redes sociais: a que aborda as negociações de Flávio Bolsonaro em defesa do fim do PIX, vista como um desmascaramento do presidenciável, e a que anuncia o vice na chapa de Renan Santos, pré-candidato à presidência pelo MBL.</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1174,215 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Dramaturgia</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>#QuemAmaCuida</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>obteve 117,4 mil depoimentos, 37% de crescimento em relação à semana anterior. Letícia Colin foi elogiada pela atuação como Adriana, personagem que virou meme e figurinha nas redes. Elisa também rendeu brincadeiras por nunca estar bem, enquanto Brigitte repercutiu após revelar a Pedro a festa de comemoração da prisão de Adriana. Parte do público ainda ironizou a torcida por casos de adultério na trama. A nova fase de Quem Ama Cuida também impulsionou as conversas no X.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dramaturgia</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#CoraçãoAcelerado</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>atingiu 6,2 mil depoimentos, significando 29% de crescimento em comparação à semana passada. O evento de Coração Acelerado em Goiânia repercutiu positivamente, com elogios aos shows de Ana Castela, Chitãozinho &amp; Xororó, Daniel e Bruno &amp; Davi. Gael também foi elogiado por seu condicionamento físico. Em contrapartida, Isadora Cruz criticou a resolução do conflito entre Agrado e Eduarda e os internautas comemoraram o fim da novela, previsto para 7 de agosto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dramaturgia</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#ANobrezadoAmor</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>registrou 4,1 mil depoimentos. Entre os destaques, a atriz Taís Araújo recebeu menções de celebração dos internautas ao serem informados de que Taís fará uma participação na novela. Houveram comentários descontraídos a respeito da duração e horário da exibição. Ainda, o perfil @forumeplay em tom informativo exibiu os pontos de audiência da novela em dias distintos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Institucional</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Institucional</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>somou 112,3 mil depoimentos. As menções de maior repercussão se desdobraram sob o contexto da Copa do Mundo. Um internauta somou 36,1 mil interações ao compartilhar um trecho da transmissão da Cazé TV onde sugeriram filmes à Globo para os horários dos jogos exclusivos, divertindo os usuários nos comentários. Além disso, a atleta Cristiane concentrou elogios do público a respeito de seus comentários durante as transmissões da TV Globo na Copa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Variedades</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#ViverSertanejo</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>alcançou 13,3 mil depoimentos, representando um crescimento de 478% em relação à semana anterior. A maior parte desses depoimentos se concentrou em menções de teor informativo a respeito da edição especial do programa em celebração dos 30 anos de 'Rei do Gado'. Além disso, o episódio que contou com a participação de Mariana Fagundes recebeu alguns elogios do público.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Variedades</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#DomingãocomHuck</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>alcançou 6,8 mil depoimentos. Usuários comentaram a respeito do 'climão' da plateia do último programa frente à eliminação da Seleção Brasileira na Copa do Mundo 2026; nesse sentido, uma internauta registrou 22,6 mil interações. Além disso, houve críticas ao programa no que tange à matéria de Lívia Andrade no apartamento de Rodrigo Branco em Miami, resultando em críticas ao apresentador Luciano Huck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Esportes</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>#CopaÉNaGlobo</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Viralizou o comentário de Ana Thaís Matos criticando Neymar durante a eliminação para a Noruega, dividindo opiniões. Receberam elogios o pedido de Caio Ribeiro para uma oportunidade ao Vozinha no futebol brasileiro e a narração de Everaldo Marques na partida contra o Japão. Por outro lado, a entrevista exclusiva da CazéTV com Cristiano Ronaldo levou parte dos internautas a comentar que a Globo estaria interessada no fim do canal no YouTube devido ao sucesso da concorrente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Esportes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>#FutebolnaGlobo</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>somou 11,7 mil depoimentos, alta de 48%.</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>somou 11,7 mil depoimentos, alta de 48% em relação à semana anterior. Perfis como @CazeTVOficial e @ESPNBrasil desejaram boa recuperação ao Luis Roberto, enquanto o @futebol_info noticiou o diagnóstico de neoplasia e divulgou o pronunciamento do narrador. Outras contas relembraram a última Copa do Mundo sem o Luis, Cléber Machado e Galvão Bueno. Perfis também comentaram a saudade do 'monopólio da Globo'. Por outro lado, houve críticas à emissora pelo uso do termo 'Brabas' para a Seleção Feminina e à redução do tempo de Três Graças por causa da transmissão do futebol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Especiais</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sessão da Tarde</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>somou 1,8 mil depoimentos. No X, a história dos sete cães que escaparam dos sequestradores e voltaram para casa gerou repercussão. Um usuário que a compartilhou descreveu o evento como 'a coisa mais filme sessão da tarde que eu já vi na vida' e alcançou 157 mil interações com seu comentário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Especiais</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>#SomBrasil</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>registrou 7,6 mil depoimentos na semana.</t>
         </is>
       </c>
     </row>
@@ -1193,11 +1397,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1206,7 +1410,7 @@
           <t>REDE</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
@@ -1218,9 +1422,9 @@
           <t>X</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>dados coletados do Twitter via Brandwatch com regras internas do time Elife</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>dados coletados do Twitter por meio do Brandwatch com regras de coleta construídas internamente pelo time Elife</t>
         </is>
       </c>
     </row>
@@ -1230,45 +1434,69 @@
           <t>Trending Topics</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Brandwatch / curadoria time Elife</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Brandwatch / Curadoria time Elife</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>hashtags oficiais + amostra de perfis</t>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>coleta do Socialnews por meio do Brandwatch, que tem como fonte páginas oficiais de perfis de notícias e influenciadores do Brasil, coletados por meio de regras booleanas construídas internamente pelo time Elife</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Socialnews / Brandwatch</t>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>coleta por meio do Brandwatch de hashtags oficiais dos produtos TVG curadas pelo time Elife, sendo que a coleta é feita somente de postagens que usam as tags, por questão de limitação da API da rede</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Instagram Public</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>coleta de posts por meio de termos de busca cadastrados do Universo TV Globo, dentro de uma amostra de 700 mil perfis de Instagram cadastrados pela Brandwatch (amostras das principais áreas de interesse: esporte, entretenimento, política, etc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>postagens e comentários</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>posts e comentários de vídeos no YouTube que citem os termos de busca cadastrados na nossa query de coleta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Depoimentos</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>volume de Twitter (tweets + RTs), Facebook (postagens e comentários do Socialnews), Instagram (postagens sem considerar comentários) e YouTube (postagens e comentários)</t>
         </is>
       </c>
     </row>
@@ -1440,11 +1668,7 @@
           <t>segunda</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>140000</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1457,11 +1681,7 @@
           <t>terça</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>86000</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1474,11 +1694,7 @@
           <t>quarta</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>100000</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1491,11 +1707,7 @@
           <t>quinta</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>95000</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1508,11 +1720,7 @@
           <t>sexta</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>74000</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1525,11 +1733,7 @@
           <t>sábado</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>72000</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1542,11 +1746,7 @@
           <t>domingo</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>146000</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1564,10 +1764,10 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1591,7 +1791,7 @@
           <t>IMAGEM_URL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>DESCRICAO</t>
         </is>
@@ -1615,20 +1815,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://twitter.com/exemplo/status/1</t>
+          <t>https://twitter.com/KleberJunco/1597753478792691713</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Descrição do post com mais engajamento no X.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>188,3 mil interações</t>
-        </is>
-      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>(preencher descrição do post — está na imagem do relatório)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1643,16 +1839,12 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Descrição do post no Instagram.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>96 mil interações</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>(preencher descrição do post)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1667,16 +1859,12 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Descrição do post no Facebook.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>54 mil interações</t>
-        </is>
-      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>(preencher descrição do post)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>